<commit_message>
Leva 1: contexto e planejamento, elemento c de G1, datas dos indicadores na ficha e estratégia da SWOT
- Processos: no G1 da pizzaria, o elemento c (critérios e indicadores)
  passa a Parcial, e o g volta a Não. Pontos 5,0 e 63% iguais; coluna c
  3 sim, 2 parcial, 4 não, como os quatro processos sem indicador. I16
  corrigido na ficha; N27 nova.
- Ficha: A1 e A3 com indicador em fevereiro de 2027, P4 e A2 em março,
  coerente com o O5 (5, 7, 9) e com a ação concluída em 10/03 (N26).
- SWOT, exemplo 2 da planilha: a estratégia W2 × O2 troca as planilhas
  pelas cotações por e-mail (N28, nova).
- testes/swot_confere_postura.py: confere a postura e as médias dos dois
  exemplos da planilha da SWOT contra a conta em Python.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Processos/Processos-modelo.xlsx
+++ b/Processos/Processos-modelo.xlsx
@@ -2016,11 +2016,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="87258834"/>
-        <c:axId val="53690365"/>
+        <c:axId val="42314841"/>
+        <c:axId val="30578834"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="87258834"/>
+        <c:axId val="42314841"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2052,7 +2052,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53690365"/>
+        <c:crossAx val="30578834"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2060,7 +2060,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="53690365"/>
+        <c:axId val="30578834"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2101,7 +2101,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87258834"/>
+        <c:crossAx val="42314841"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -2267,11 +2267,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="339729"/>
-        <c:axId val="40387945"/>
+        <c:axId val="47195182"/>
+        <c:axId val="7637829"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="339729"/>
+        <c:axId val="47195182"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2303,7 +2303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40387945"/>
+        <c:crossAx val="7637829"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2311,7 +2311,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40387945"/>
+        <c:axId val="7637829"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2352,7 +2352,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="339729"/>
+        <c:crossAx val="47195182"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -4656,13 +4656,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
+    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H4" type="date">
+      <formula1>36526</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Digite um número inteiro de 1 a 12." errorStyle="stop" errorTitle="Número inválido" operator="between" prompt="Número do processo, como na aba Processos." promptTitle="Número" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D4" type="whole">
       <formula1>1</formula1>
       <formula2>12</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H4" type="date">
-      <formula1>36526</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
@@ -5967,7 +5967,7 @@
         <v>160</v>
       </c>
       <c r="J11" s="40" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K11" s="40" t="s">
         <v>159</v>
@@ -5979,7 +5979,7 @@
         <v>160</v>
       </c>
       <c r="N11" s="40" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="O11" s="40" t="s">
         <v>160</v>
@@ -6428,7 +6428,7 @@
       </c>
       <c r="J20" s="35" t="n">
         <f aca="false">(COUNTIF(J11:J19,"Sim")+0.5*COUNTIF(J11:J19,"Parcial"))/ROWS(J11:J19)</f>
-        <v>0.388888888888889</v>
+        <v>0.444444444444444</v>
       </c>
       <c r="K20" s="35" t="n">
         <f aca="false">(COUNTIF(K11:K19,"Sim")+0.5*COUNTIF(K11:K19,"Parcial"))/ROWS(K11:K19)</f>
@@ -6444,7 +6444,7 @@
       </c>
       <c r="N20" s="35" t="n">
         <f aca="false">(COUNTIF(N11:N19,"Sim")+0.5*COUNTIF(N11:N19,"Parcial"))/ROWS(N11:N19)</f>
-        <v>0.388888888888889</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="O20" s="35" t="n">
         <f aca="false">(COUNTIF(O11:O19,"Sim")+0.5*COUNTIF(O11:O19,"Parcial"))/ROWS(O11:O19)</f>
@@ -6551,7 +6551,7 @@
       <c r="D28" s="22"/>
       <c r="E28" s="23" t="str">
         <f aca="false">INDEX(H10:O10,MATCH(MIN(H20:O20),H20:O20,0))</f>
-        <v>c · Critérios e indicadores</v>
+        <v>g · Avaliação e mudanças</v>
       </c>
       <c r="F28" s="23"/>
       <c r="G28" s="23"/>

</xml_diff>